<commit_message>
Paid membership: Stripe checkout, email sign-in, member home, numbers on the map and property pages
Cloudflare Pages Functions (functions/api, lib/members.js) with one KV namespace (MEMBERS).
Stays closed until the Stripe keys and the KV binding are set (README, Membership).
Member data is built by the daily refresh in the runner's temp folder and uploaded keyless
(GitHub OIDC), never written to site/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/free-list/first-tuesday-list-2026-11-03.xlsx
+++ b/site/free-list/first-tuesday-list-2026-11-03.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Nov 3, 2026 sale" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nov 3, 2026 sale" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nov 3, 2026 sale'!$A$4:$P$799</definedName>
@@ -281,7 +281,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -296,13 +296,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -311,7 +311,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -326,13 +326,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>